<commit_message>
Clearer planning status, resilience fixes and macOS launcher
- Split "behind plan" into late start (go-live still possible) and
  missed go-live; Coming up shows the next deadline with a day count.
- window() includes ranges that started the previous year.
- Campaigns whose moment no longer exists are skipped with a warning
  instead of breaking pages, so they can still be removed.
- run_app.command for macOS; screenshots and examples regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/seasonsignal-2026-food-fjellbrus-demo.xlsx
+++ b/examples/seasonsignal-2026-food-fjellbrus-demo.xlsx
@@ -2172,7 +2172,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>behind plan</t>
+          <t>late start</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">

</xml_diff>

<commit_message>
All app text in English; no built-in data limits
Moments show their English name with the Norwegian name in brackets on
screen and in the XLSX and ICS exports; regions, notes and screen texts
gloss Norwegian terms on first use. The demo stays Norwegian with a note.
Season Signal has no upload, so it has no data limits locally or in a
public demo; launchers and Docker default to the suite's 10,000 MB cap.
Example calendars regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/seasonsignal-2026-food-fjellbrus-demo.xlsx
+++ b/examples/seasonsignal-2026-food-fjellbrus-demo.xlsx
@@ -434,26 +434,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
     <col width="60" customWidth="1" min="15" max="15"/>
     <col width="60" customWidth="1" min="16" max="16"/>
-    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,80 +463,75 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Moment (en)</t>
+          <t>Kind</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Kind</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Start</t>
+          <t>End</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>End</t>
+          <t>Varies locally</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Varies locally</t>
+          <t>Region</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Region</t>
+          <t>Categories</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Categories</t>
+          <t>Concept &amp; brief</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Concept &amp; brief</t>
+          <t>Creative production</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Creative production</t>
+          <t>Media booking</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Media booking</t>
+          <t>Campaign live</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Campaign live</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Basis</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Basis</t>
+          <t>Rule</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Rule</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -546,211 +540,196 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nyttårsdag</t>
+          <t>New Year's Day (Nyttårsdag)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New Year's Day</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46023</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>46023</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, B2B</t>
         </is>
       </c>
+      <c r="H2" s="2" t="n">
+        <v>45911</v>
+      </c>
       <c r="I2" s="2" t="n">
-        <v>45911</v>
+        <v>45953</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>45953</v>
+        <v>45981</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>45981</v>
-      </c>
-      <c r="L2" s="2" t="n">
         <v>46015</v>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>1 Jan</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1 Jan</t>
+          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Helligdag under helligdagsfredloven § 2. "New year, new me" — health, fitness and budgeting messages.</t>
+          <t>Public holiday (helligdag) under the Public Holidays Act (helligdagsfredloven) § 2. "New year, new me" — health, fitness and budgeting messages.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tørrlagt januar (Dry January)</t>
+          <t>Dry January (Tørrlagt januar)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dry January</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
           <t>Cultural moment</t>
         </is>
       </c>
+      <c r="C3" s="2" t="n">
+        <v>46023</v>
+      </c>
       <c r="D3" s="2" t="n">
-        <v>46023</v>
-      </c>
-      <c r="E3" s="2" t="n">
         <v>46053</v>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>Alcohol-free, Food &amp; drink</t>
         </is>
       </c>
+      <c r="H3" s="2" t="n">
+        <v>45911</v>
+      </c>
       <c r="I3" s="2" t="n">
-        <v>45911</v>
+        <v>45953</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>45953</v>
+        <v>45981</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>45981</v>
-      </c>
-      <c r="L3" s="2" t="n">
         <v>46015</v>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>1 Jan → 31 Jan</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>1 Jan → 31 Jan</t>
+          <t>https://alcoholchange.org.uk/get-involved/campaigns/dry-january</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>https://alcoholchange.org.uk/get-involved/campaigns/dry-january</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>International campaign month, widely picked up in Norway. No Norwegian owner. Remember that alcohol advertising is banned in Norway (alkoholloven § 9-2); alcohol-free variants need care not to promote the parent brand.</t>
+          <t>International campaign month, widely picked up in Norway. No Norwegian owner. Remember that alcohol advertising is banned in Norway (the Alcohol Act, alkoholloven § 9-2); alcohol-free variants need care not to promote the parent brand.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Morsdag</t>
+          <t>Mother's Day, Norway (Morsdag)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mother's Day (Norway)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
           <t>Retail moment</t>
         </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>46061</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>46061</v>
       </c>
-      <c r="E4" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, Fashion, Kids &amp; family</t>
         </is>
       </c>
+      <c r="H4" s="2" t="n">
+        <v>45947</v>
+      </c>
       <c r="I4" s="2" t="n">
-        <v>45947</v>
+        <v>45989</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>45989</v>
+        <v>46015</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>46015</v>
-      </c>
-      <c r="L4" s="2" t="n">
         <v>46052</v>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>tradition</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>tradition</t>
+          <t>2nd sun of Feb</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2nd sun of Feb</t>
+          <t>https://snl.no/morsdag</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
-        <is>
-          <t>https://snl.no/morsdag</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
         <is>
           <t>Second Sunday in FEBRUARY in Norway (not May as in the US/most of Europe). Flowers, chocolate, breakfast-in-bed. International brands regularly get this wrong.</t>
         </is>
@@ -759,1146 +738,1066 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Valentinsdagen</t>
+          <t>Valentine's Day (Valentinsdagen)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Valentine's Day</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
           <t>Retail moment</t>
         </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>46067</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>46067</v>
       </c>
-      <c r="E5" s="2" t="n">
-        <v>46067</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, Fashion</t>
         </is>
       </c>
+      <c r="H5" s="2" t="n">
+        <v>45954</v>
+      </c>
       <c r="I5" s="2" t="n">
-        <v>45954</v>
+        <v>45996</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>45996</v>
+        <v>46024</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>46024</v>
-      </c>
-      <c r="L5" s="2" t="n">
         <v>46059</v>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>14 Feb</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>14 Feb</t>
+          <t>https://snl.no/valentinsdag</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://snl.no/valentinsdag</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Imported convention; fixed date. Often within days of morsdag — plan the two together.</t>
+          <t>Imported convention; fixed date. Often within days of Mother's Day (morsdag) — plan the two together.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fastelavnssøndag</t>
+          <t>Shrovetide Sunday (Fastelavnssøndag)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Shrovetide Sunday</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
           <t>Cultural moment</t>
         </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>46068</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>46068</v>
       </c>
-      <c r="E6" s="2" t="n">
-        <v>46068</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
           <t>Food &amp; drink, Kids &amp; family</t>
         </is>
       </c>
+      <c r="H6" s="2" t="n">
+        <v>45954</v>
+      </c>
       <c r="I6" s="2" t="n">
-        <v>45954</v>
+        <v>45996</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>45996</v>
+        <v>46024</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>46024</v>
-      </c>
-      <c r="L6" s="2" t="n">
         <v>46059</v>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>tradition</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>tradition</t>
+          <t>Easter Sunday − 49 d</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Easter Sunday − 49 d</t>
+          <t>https://snl.no/fastelavn</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>https://snl.no/fastelavn</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Easter Sunday − 49 days (falls 1 Feb – 7 Mar). Fastelavnsboller with cream; fastelavnsris.</t>
+          <t>Easter Sunday − 49 days (falls 1 Feb – 7 Mar). Shrovetide buns (fastelavnsboller) with cream; decorated birch twigs (fastelavnsris).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Vinterferie</t>
+          <t>Winter school break (Vinterferie)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Winter school break</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
           <t>Season &amp; holidays</t>
         </is>
       </c>
+      <c r="C7" s="2" t="n">
+        <v>46069</v>
+      </c>
       <c r="D7" s="2" t="n">
-        <v>46069</v>
-      </c>
-      <c r="E7" s="2" t="n">
         <v>46080</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Yes — range</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Yes — range</t>
+          <t>All of Norway</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
           <t>Travel, Kids &amp; family, Food &amp; drink, Retail</t>
         </is>
       </c>
+      <c r="H7" s="2" t="n">
+        <v>45957</v>
+      </c>
       <c r="I7" s="2" t="n">
-        <v>45957</v>
+        <v>45999</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>45999</v>
+        <v>46027</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>46027</v>
-      </c>
-      <c r="L7" s="2" t="n">
         <v>46062</v>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>observed</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>observed</t>
+          <t>mon of ISO week 8 → fri of ISO week 9</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>mon of ISO week 8 → fri of ISO week 9</t>
+          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>One school week in ISO week 8 OR 9, set locally (kommune for grunnskole, fylkeskommune for vgs) under opplæringslova § 14-1. The national entry spans both weeks — check the local skolerute.</t>
+          <t>One school week in ISO week 8 OR 9, set locally (by the municipality, kommune, for primary and lower-secondary school; by the county, fylkeskommune, for upper-secondary school) under the Education Act (opplæringslova) § 14-1. The national entry spans both weeks — check the local school calendar (skolerute).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Påskeferie</t>
+          <t>Easter school break (Påskeferie)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Easter school break</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
           <t>Season &amp; holidays</t>
         </is>
       </c>
+      <c r="C8" s="2" t="n">
+        <v>46109</v>
+      </c>
       <c r="D8" s="2" t="n">
-        <v>46109</v>
-      </c>
-      <c r="E8" s="2" t="n">
         <v>46119</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Yes — range</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Yes — range</t>
+          <t>All of Norway</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
           <t>Travel, Food &amp; drink, Kids &amp; family, Retail, Alcohol-free</t>
         </is>
       </c>
+      <c r="H8" s="2" t="n">
+        <v>45996</v>
+      </c>
       <c r="I8" s="2" t="n">
-        <v>45996</v>
+        <v>46038</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>46038</v>
+        <v>46066</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>46066</v>
-      </c>
-      <c r="L8" s="2" t="n">
         <v>46101</v>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>observed</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>observed</t>
+          <t>Easter Sunday − 8 d → Easter Sunday + 2 d</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Easter Sunday − 8 d → Easter Sunday + 2 d</t>
+          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>Schools close from the Monday before skjærtorsdag through 2. påskedag; some kommuner add the Tuesday. Range shown: Saturday before palmesøndag to Easter Tuesday. Peak cabin and mountain season.</t>
+          <t>Schools close from the Monday before Maundy Thursday through Easter Monday; some municipalities (kommuner) add the Tuesday. Range shown: Saturday before Palm Sunday to Easter Tuesday. Peak cabin and mountain season.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Skjærtorsdag</t>
+          <t>Maundy Thursday (Skjærtorsdag)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Maundy Thursday</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>46114</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>46114</v>
       </c>
-      <c r="E9" s="2" t="n">
-        <v>46114</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, Travel, Alcohol-free</t>
         </is>
       </c>
+      <c r="H9" s="2" t="n">
+        <v>46002</v>
+      </c>
       <c r="I9" s="2" t="n">
-        <v>46002</v>
+        <v>46044</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>46044</v>
+        <v>46072</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>46072</v>
-      </c>
-      <c r="L9" s="2" t="n">
         <v>46107</v>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>Easter Sunday − 3 d</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Easter Sunday − 3 d</t>
+          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>Helligdag; Easter Sunday − 3 days. Most shops closed — last grocery run is Wednesday.</t>
+          <t>Public holiday (helligdag); Easter Sunday − 3 days. Most shops closed — last grocery run is Wednesday.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Langfredag</t>
+          <t>Good Friday (Langfredag)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Good Friday</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>46115</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>46115</v>
       </c>
-      <c r="E10" s="2" t="n">
-        <v>46115</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
           <t>Food &amp; drink, Travel</t>
         </is>
       </c>
+      <c r="H10" s="2" t="n">
+        <v>46003</v>
+      </c>
       <c r="I10" s="2" t="n">
-        <v>46003</v>
+        <v>46045</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>46045</v>
+        <v>46073</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>46073</v>
-      </c>
-      <c r="L10" s="2" t="n">
         <v>46108</v>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>Easter Sunday − 2 d</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Easter Sunday − 2 d</t>
+          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>Helligdag; Easter Sunday − 2 days.</t>
+          <t>Public holiday (helligdag); Easter Sunday − 2 days.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Påskedag</t>
+          <t>Easter Sunday (Påskedag)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Easter Sunday</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>46117</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>46117</v>
       </c>
-      <c r="E11" s="2" t="n">
-        <v>46117</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, Travel, Kids &amp; family, Alcohol-free</t>
         </is>
       </c>
+      <c r="H11" s="2" t="n">
+        <v>46003</v>
+      </c>
       <c r="I11" s="2" t="n">
-        <v>46003</v>
+        <v>46045</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>46045</v>
+        <v>46073</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>46073</v>
-      </c>
-      <c r="L11" s="2" t="n">
         <v>46108</v>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>Easter Sunday</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Easter Sunday</t>
+          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>Helligdag; Western Easter (first Sunday after the first full moon on or after 21 March, as defined in the law). Påskeegg, påskekrim, cabin trips.</t>
+          <t>Helligdag; Western Easter (first Sunday after the first full moon on or after 21 March, as defined in the law). Easter eggs (påskeegg), Easter crime fiction (påskekrim), cabin trips.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2. påskedag</t>
+          <t>Easter Monday (2. påskedag)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Easter Monday</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>46118</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>46118</v>
       </c>
-      <c r="E12" s="2" t="n">
-        <v>46118</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
           <t>Travel</t>
         </is>
       </c>
+      <c r="H12" s="2" t="n">
+        <v>46006</v>
+      </c>
       <c r="I12" s="2" t="n">
-        <v>46006</v>
+        <v>46048</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>46048</v>
+        <v>46076</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>46076</v>
-      </c>
-      <c r="L12" s="2" t="n">
         <v>46111</v>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>Easter Sunday + 1 d</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Easter Sunday + 1 d</t>
+          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>Helligdag; Easter Sunday + 1 day. Return-traffic day from the cabin.</t>
+          <t>Public holiday (helligdag); Easter Sunday + 1 day. Return-traffic day from the cabin.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Russetiden</t>
+          <t>Russ celebration season (Russetiden)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Russ celebration season</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
           <t>Season &amp; holidays</t>
         </is>
       </c>
+      <c r="C13" s="2" t="n">
+        <v>46132</v>
+      </c>
       <c r="D13" s="2" t="n">
-        <v>46132</v>
-      </c>
-      <c r="E13" s="2" t="n">
         <v>46159</v>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
           <t>Fashion, Food &amp; drink, Retail, Alcohol-free</t>
         </is>
       </c>
+      <c r="H13" s="2" t="n">
+        <v>46020</v>
+      </c>
       <c r="I13" s="2" t="n">
-        <v>46020</v>
+        <v>46062</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>46062</v>
+        <v>46090</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>46090</v>
-      </c>
-      <c r="L13" s="2" t="n">
         <v>46125</v>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>20 Apr → 17 May</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>20 Apr → 17 May</t>
+          <t>https://www.regjeringen.no/no/aktuelt/regjeringen-skal-endre-russetiden/id3030864/</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>https://www.regjeringen.no/no/aktuelt/regjeringen-skal-endre-russetiden/id3030864/</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>Traditionally ~20 April to 17. mai for final-year upper-secondary students (russ). No legal dates. The Government aims to move the celebration after exams and from 2026 spreads vg3 written exams either side of 17. mai — expect this window to shift; re-check each year. Marketing to russ involves minors: avoid alcohol and pressure tactics.</t>
+          <t>Traditionally ~20 April to 17. mai for final-year upper-secondary students (russ). No legal dates. The Government aims to move the celebration after exams and from 2026 spreads final-year (vg3) written exams either side of 17. mai — expect this window to shift; re-check each year. Marketing to russ involves minors: avoid alcohol and pressure tactics.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1. mai — Arbeidernes dag</t>
+          <t>May Day (1. mai — Arbeidernes dag)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>May Day</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>46143</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>46143</v>
       </c>
-      <c r="E14" s="2" t="n">
-        <v>46143</v>
-      </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
           <t>B2B</t>
         </is>
       </c>
+      <c r="H14" s="2" t="n">
+        <v>46031</v>
+      </c>
       <c r="I14" s="2" t="n">
-        <v>46031</v>
+        <v>46073</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>46073</v>
+        <v>46101</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>46101</v>
-      </c>
-      <c r="L14" s="2" t="n">
         <v>46136</v>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>1 May</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>1 May</t>
+          <t>https://lovdata.no/dokument/NL/lov/1947-04-26-1</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1947-04-26-1</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>Offentlig høytidsdag under lov om 1. og 17. mai som høgtidsdager.</t>
+          <t>Official public holiday under the Act on 1 and 17 May as public holidays (lov om 1. og 17. mai som høgtidsdager).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Kristi himmelfartsdag</t>
+          <t>Ascension Day (Kristi himmelfartsdag)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ascension Day</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>46156</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>46156</v>
       </c>
-      <c r="E15" s="2" t="n">
-        <v>46156</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
           <t>Travel, Retail</t>
         </is>
       </c>
+      <c r="H15" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="I15" s="2" t="n">
-        <v>46044</v>
+        <v>46086</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>46086</v>
+        <v>46113</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>46113</v>
-      </c>
-      <c r="L15" s="2" t="n">
         <v>46149</v>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>Easter Sunday + 39 d</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Easter Sunday + 39 d</t>
+          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>Helligdag; Easter Sunday + 39 days (always a Thursday). Many take Friday off — a long weekend.</t>
+          <t>Public holiday (helligdag); Easter Sunday + 39 days (always a Thursday). Many take Friday off — a long weekend.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>17. mai — Grunnlovsdagen</t>
+          <t>Constitution Day (17. mai — Grunnlovsdagen)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Constitution Day</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>46159</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>46159</v>
       </c>
-      <c r="E16" s="2" t="n">
-        <v>46159</v>
-      </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, Fashion, Kids &amp; family, Alcohol-free</t>
         </is>
       </c>
+      <c r="H16" s="2" t="n">
+        <v>46045</v>
+      </c>
       <c r="I16" s="2" t="n">
-        <v>46045</v>
+        <v>46087</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>46087</v>
+        <v>46113</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>46113</v>
-      </c>
-      <c r="L16" s="2" t="n">
         <v>46150</v>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>17 May</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>17 May</t>
+          <t>https://lovdata.no/dokument/NL/lov/1947-04-26-1</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1947-04-26-1</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>Offentlig høytidsdag (lov om 1. og 17. mai som høgtidsdager). Norway's biggest food, ice-cream, sausage, bunad and party-wear moment; also the end of russetid.</t>
+          <t>Official public holiday (Act on 1 and 17 May as public holidays, lov om 1. og 17. mai som høgtidsdager). Norway's biggest food, ice-cream, sausage, bunad (national costume) and party-wear moment; also the end of the russ season (russetid).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pinsedag</t>
+          <t>Whit Sunday (Pinsedag)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Whit Sunday</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>46166</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>46166</v>
       </c>
-      <c r="E17" s="2" t="n">
-        <v>46166</v>
-      </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
           <t>Travel</t>
         </is>
       </c>
+      <c r="H17" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="I17" s="2" t="n">
-        <v>46052</v>
+        <v>46094</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>46094</v>
+        <v>46122</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>46122</v>
-      </c>
-      <c r="L17" s="2" t="n">
         <v>46157</v>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>Easter Sunday + 49 d</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Easter Sunday + 49 d</t>
+          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>Helligdag; Easter Sunday + 49 days.</t>
+          <t>Public holiday (helligdag); Easter Sunday + 49 days.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2. pinsedag</t>
+          <t>Whit Monday (2. pinsedag)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Whit Monday</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>46167</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>46167</v>
       </c>
-      <c r="E18" s="2" t="n">
-        <v>46167</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
           <t>Travel, Retail</t>
         </is>
       </c>
+      <c r="H18" s="2" t="n">
+        <v>46055</v>
+      </c>
       <c r="I18" s="2" t="n">
-        <v>46055</v>
+        <v>46097</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>46097</v>
+        <v>46125</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>46125</v>
-      </c>
-      <c r="L18" s="2" t="n">
         <v>46160</v>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>Easter Sunday + 50 d</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Easter Sunday + 50 d</t>
+          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>Helligdag; Easter Sunday + 50 days. Long weekend; often the first garden/grill weekend.</t>
+          <t>Public holiday (helligdag); Easter Sunday + 50 days. Long weekend; often the first garden/grill weekend.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Skoleslutt</t>
+          <t>Last day of school (Skoleslutt)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Last day of school</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
           <t>Season &amp; holidays</t>
         </is>
       </c>
+      <c r="C19" s="2" t="n">
+        <v>46190</v>
+      </c>
       <c r="D19" s="2" t="n">
-        <v>46190</v>
-      </c>
-      <c r="E19" s="2" t="n">
         <v>46197</v>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Yes — range</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Yes — range</t>
+          <t>All of Norway</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
           <t>Kids &amp; family, Retail, Travel, Food &amp; drink</t>
         </is>
       </c>
+      <c r="H19" s="2" t="n">
+        <v>46078</v>
+      </c>
       <c r="I19" s="2" t="n">
-        <v>46078</v>
+        <v>46120</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>46120</v>
+        <v>46148</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>46148</v>
-      </c>
-      <c r="L19" s="2" t="n">
         <v>46183</v>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>observed</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>observed</t>
+          <t>17 Jun → 24 Jun</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>17 Jun → 24 Jun</t>
+          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>Set in each kommune's skolerute (opplæringslova § 14-1); usually a weekday between ~17 and 24 June. Oslo's last day was Fri 18 June 2027 and is Thu 22 June 2028 — no stable weekday rule, so a range.</t>
+          <t>Set in each municipality's school calendar (skolerute; opplæringslova § 14-1); usually a weekday between ~17 and 24 June. Oslo's last day was Fri 18 June 2027 and is Thu 22 June 2028 — no stable weekday rule, so a range.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sankthansaften</t>
+          <t>Midsummer Eve (Sankthansaften)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Midsummer Eve</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
           <t>Cultural moment</t>
         </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>46196</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>46196</v>
       </c>
-      <c r="E20" s="2" t="n">
-        <v>46196</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
           <t>Food &amp; drink, Alcohol-free</t>
         </is>
       </c>
+      <c r="H20" s="2" t="n">
+        <v>46084</v>
+      </c>
       <c r="I20" s="2" t="n">
-        <v>46084</v>
+        <v>46126</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>46126</v>
+        <v>46154</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>46154</v>
-      </c>
-      <c r="L20" s="2" t="n">
         <v>46189</v>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>tradition</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>tradition</t>
+          <t>23 Jun</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>23 Jun</t>
+          <t>https://snl.no/sankthans</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
-        <is>
-          <t>https://snl.no/sankthans</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
         <is>
           <t>Bonfires and grilling on 23 June; not a public holiday (SNL).</t>
         </is>
@@ -1907,219 +1806,204 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Fellesferie</t>
+          <t>Collective summer holiday (Fellesferie)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Collective summer holiday</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
           <t>Season &amp; holidays</t>
         </is>
       </c>
+      <c r="C21" s="2" t="n">
+        <v>46209</v>
+      </c>
       <c r="D21" s="2" t="n">
-        <v>46209</v>
-      </c>
-      <c r="E21" s="2" t="n">
         <v>46227</v>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
           <t>Travel, Food &amp; drink, Retail, B2B, Alcohol-free</t>
         </is>
       </c>
+      <c r="H21" s="2" t="n">
+        <v>46097</v>
+      </c>
       <c r="I21" s="2" t="n">
-        <v>46097</v>
+        <v>46139</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>46139</v>
+        <v>46164</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>46164</v>
-      </c>
-      <c r="L21" s="2" t="n">
         <v>46202</v>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>mon of ISO week 28 → fri of ISO week 30</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>mon of ISO week 28 → fri of ISO week 30</t>
+          <t>https://www.thelocal.no/20210702/fellesferie-everything-you-need-to-know-about-norways-collective-holiday-period</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>https://www.thelocal.no/20210702/fellesferie-everything-you-need-to-know-about-norways-collective-holiday-period</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>Traditionally ISO weeks 28–30 in July, recommended by NHO and Fellesforbundet for industry (6–24 July in 2026). Ferieloven § 5 lets employees claim 3 weeks' main holiday between 1 June and 30 September (https://lovdata.no/dokument/NL/lov/1988-04-29-21). B2B goes quiet; travel, grilling and cabin peak.</t>
+          <t>Traditionally ISO weeks 28–30 in July, recommended by NHO (the Confederation of Norwegian Enterprise) and Fellesforbundet (the United Federation of Trade Unions) for industry (6–24 July in 2026). The Holidays Act (ferieloven) § 5 lets employees claim 3 weeks' main holiday between 1 June and 30 September (https://lovdata.no/dokument/NL/lov/1988-04-29-21). B2B goes quiet; travel, grilling and cabin peak.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Skolestart</t>
+          <t>Back to school (Skolestart)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Back to school</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
           <t>Season &amp; holidays</t>
         </is>
       </c>
+      <c r="C22" s="2" t="n">
+        <v>46244</v>
+      </c>
       <c r="D22" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="E22" s="2" t="n">
         <v>46255</v>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Yes — range</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Yes — range</t>
+          <t>All of Norway</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
           <t>Kids &amp; family, Retail, Fashion, Food &amp; drink, B2B</t>
         </is>
       </c>
+      <c r="H22" s="2" t="n">
+        <v>46132</v>
+      </c>
       <c r="I22" s="2" t="n">
-        <v>46132</v>
+        <v>46174</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>46174</v>
+        <v>46202</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>46202</v>
-      </c>
-      <c r="L22" s="2" t="n">
         <v>46237</v>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>passed</t>
+          <t>observed</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>observed</t>
+          <t>mon of ISO week 33 → fri of ISO week 34</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>mon of ISO week 33 → fri of ISO week 34</t>
+          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>First school day is set locally, usually mid-August (ISO week 33 or 34) — Bergen even varies the weekday (Fri 14 Aug 2026, Mon 16 Aug 2027), so it keeps the national range. Back-to-school is also "høstoppstart" for B2B: offices fill up again after fellesferie.</t>
+          <t>First school day is set locally, usually mid-August (ISO week 33 or 34) — Bergen even varies the weekday (Fri 14 Aug 2026, Mon 16 Aug 2027), so it keeps the national range. Back-to-school is also the autumn restart ("høstoppstart") for B2B: offices fill up again after the collective summer holiday (fellesferie).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Høstferie</t>
+          <t>Autumn school break (Høstferie)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Autumn school break</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
           <t>Season &amp; holidays</t>
         </is>
       </c>
+      <c r="C23" s="2" t="n">
+        <v>46293</v>
+      </c>
       <c r="D23" s="2" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E23" s="2" t="n">
         <v>46304</v>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Yes — range</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Yes — range</t>
+          <t>All of Norway</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
           <t>Travel, Kids &amp; family, Food &amp; drink</t>
         </is>
       </c>
+      <c r="H23" s="2" t="n">
+        <v>46181</v>
+      </c>
       <c r="I23" s="2" t="n">
-        <v>46181</v>
+        <v>46223</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>46223</v>
+        <v>46251</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="L23" s="2" t="n">
         <v>46286</v>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>happening now</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>happening now</t>
+          <t>observed</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>observed</t>
+          <t>mon of ISO week 40 → fri of ISO week 41</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>mon of ISO week 40 → fri of ISO week 41</t>
+          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
-        <is>
-          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
         <is>
           <t>One school week in ISO week 40 or 41, set locally (e.g. Oslo and Bærum week 40; Trondheim, Haugesund and Nord-Aurdal week 41 in 2026). The national entry spans both weeks.</t>
         </is>
@@ -2133,64 +2017,59 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Halloween</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
           <t>Retail moment</t>
         </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>46326</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>46326</v>
       </c>
-      <c r="E24" s="2" t="n">
-        <v>46326</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, Kids &amp; family, Fashion</t>
         </is>
       </c>
+      <c r="H24" s="2" t="n">
+        <v>46213</v>
+      </c>
       <c r="I24" s="2" t="n">
-        <v>46213</v>
+        <v>46255</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>46255</v>
+        <v>46283</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L24" s="2" t="n">
         <v>46318</v>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>31 Oct</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>31 Oct</t>
+          <t>https://snl.no/halloween</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
-        <is>
-          <t>https://snl.no/halloween</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
         <is>
           <t>Imported convention, now a significant sweets and costume moment. Fixed date.</t>
         </is>
@@ -2199,69 +2078,64 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Farsdag</t>
+          <t>Father's Day, Norway (Farsdag)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Father's Day (Norway)</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
           <t>Retail moment</t>
         </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>46334</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>46334</v>
       </c>
-      <c r="E25" s="2" t="n">
-        <v>46334</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, Fashion, Kids &amp; family</t>
         </is>
       </c>
+      <c r="H25" s="2" t="n">
+        <v>46220</v>
+      </c>
       <c r="I25" s="2" t="n">
-        <v>46220</v>
+        <v>46262</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>46262</v>
+        <v>46290</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>46290</v>
-      </c>
-      <c r="L25" s="2" t="n">
         <v>46325</v>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>tradition</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>tradition</t>
+          <t>2nd sun of Nov</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2nd sun of Nov</t>
+          <t>https://snl.no/farsdag</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
-        <is>
-          <t>https://snl.no/farsdag</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
         <is>
           <t>Second Sunday in NOVEMBER in Norway (not June as in the US/UK). Lands just before Black Week.</t>
         </is>
@@ -2270,69 +2144,64 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Julebordsesongen</t>
+          <t>Christmas-party season (Julebordsesongen)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Christmas-party season</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
           <t>Cultural moment</t>
         </is>
       </c>
+      <c r="C26" s="2" t="n">
+        <v>46339</v>
+      </c>
       <c r="D26" s="2" t="n">
-        <v>46339</v>
-      </c>
-      <c r="E26" s="2" t="n">
         <v>46375</v>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
           <t>Food &amp; drink, Fashion, B2B, Alcohol-free</t>
         </is>
       </c>
+      <c r="H26" s="2" t="n">
+        <v>46227</v>
+      </c>
       <c r="I26" s="2" t="n">
-        <v>46227</v>
+        <v>46269</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>46269</v>
+        <v>46297</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>46297</v>
-      </c>
-      <c r="L26" s="2" t="n">
         <v>46332</v>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>2nd fri of Nov → 3rd sat of Dec</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2nd fri of Nov → 3rd sat of Dec</t>
+          <t>https://snl.no/julebord</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
-        <is>
-          <t>https://snl.no/julebord</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
         <is>
           <t>Workplace Christmas parties cluster on Friday/Saturday evenings from mid-November to mid-December. No official dates; the range is a planning convention. Venues book up by early autumn.</t>
         </is>
@@ -2346,64 +2215,59 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Black Week</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
           <t>Retail moment</t>
         </is>
       </c>
+      <c r="C27" s="2" t="n">
+        <v>46349</v>
+      </c>
       <c r="D27" s="2" t="n">
-        <v>46349</v>
-      </c>
-      <c r="E27" s="2" t="n">
         <v>46356</v>
       </c>
-      <c r="F27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
           <t>Retail, Fashion, Food &amp; drink, Kids &amp; family</t>
         </is>
       </c>
+      <c r="H27" s="2" t="n">
+        <v>46237</v>
+      </c>
       <c r="I27" s="2" t="n">
-        <v>46237</v>
+        <v>46279</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>46279</v>
+        <v>46307</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L27" s="2" t="n">
         <v>46342</v>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>start of 'black_friday' − 4 d → start of 'black_friday' + 3 d</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>start of 'black_friday' − 4 d → start of 'black_friday' + 3 d</t>
+          <t>https://www.bi.no/forskning/business-review/articles/2021/11/gi-norske-forbrukere-en-gronnere-black-friday/</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
-        <is>
-          <t>https://www.bi.no/forskning/business-review/articles/2021/11/gi-norske-forbrukere-en-gronnere-black-friday/</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
         <is>
           <t>Norwegian retailers stretch Black Friday into a week — commonly Monday of Black Friday week through Cyber Monday. Many start earlier ("Black November"); treat the start as the latest safe go-live.</t>
         </is>
@@ -2412,71 +2276,66 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Julehandelen</t>
+          <t>Christmas shopping season (Julehandelen)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Christmas shopping season</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
           <t>Retail moment</t>
         </is>
       </c>
+      <c r="C28" s="2" t="n">
+        <v>46349</v>
+      </c>
       <c r="D28" s="2" t="n">
-        <v>46349</v>
-      </c>
-      <c r="E28" s="2" t="n">
         <v>46380</v>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, Fashion, Kids &amp; family, Alcohol-free</t>
         </is>
       </c>
+      <c r="H28" s="2" t="n">
+        <v>46237</v>
+      </c>
       <c r="I28" s="2" t="n">
-        <v>46237</v>
+        <v>46279</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>46279</v>
+        <v>46307</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>46307</v>
-      </c>
-      <c r="L28" s="2" t="n">
         <v>46342</v>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>start of 'black_week' → 24 Dec</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>start of 'black_week' → 24 Dec</t>
+          <t>https://www.virke.no/analyse/julehandel/</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>https://www.virke.no/analyse/julehandel/</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>Retail's peak season. Now effectively starts with Black Week and runs to julaften; Virke reports November + December as the julehandel period.</t>
+          <t>Retail's peak season. Now effectively starts with Black Week and runs to Christmas Eve (julaften); Virke (the Federation of Norwegian Enterprise) reports November + December as the Christmas shopping (julehandel) period.</t>
         </is>
       </c>
     </row>
@@ -2488,64 +2347,59 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Black Friday</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
           <t>Retail moment</t>
         </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>46353</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>46353</v>
       </c>
-      <c r="E29" s="2" t="n">
-        <v>46353</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
           <t>Retail, Fashion, Food &amp; drink, B2B</t>
         </is>
       </c>
+      <c r="H29" s="2" t="n">
+        <v>46241</v>
+      </c>
       <c r="I29" s="2" t="n">
-        <v>46241</v>
+        <v>46283</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>46283</v>
+        <v>46311</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>46311</v>
-      </c>
-      <c r="L29" s="2" t="n">
         <v>46346</v>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>4th thu of Nov + 1 d</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>4th thu of Nov + 1 d</t>
+          <t>https://snl.no/Black_Friday</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
-        <is>
-          <t>https://snl.no/Black_Friday</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
         <is>
           <t>The day after US Thanksgiving (4th Thursday of November + 1). Imported convention; Norway's single biggest online-retail day.</t>
         </is>
@@ -2554,69 +2408,64 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1. søndag i advent</t>
+          <t>First Sunday of Advent (1. søndag i advent)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>First Sunday of Advent</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
           <t>Cultural moment</t>
         </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>46355</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>46355</v>
       </c>
-      <c r="E30" s="2" t="n">
-        <v>46355</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, Kids &amp; family</t>
         </is>
       </c>
+      <c r="H30" s="2" t="n">
+        <v>46241</v>
+      </c>
       <c r="I30" s="2" t="n">
-        <v>46241</v>
+        <v>46283</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>46283</v>
+        <v>46311</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>46311</v>
-      </c>
-      <c r="L30" s="2" t="n">
         <v>46346</v>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>tradition</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>tradition</t>
+          <t>first sun on/after 27 Nov</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>first sun on/after 27 Nov</t>
+          <t>https://snl.no/advent</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
-        <is>
-          <t>https://snl.no/advent</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
         <is>
           <t>Four Sundays before Christmas Day; always 27 Nov – 3 Dec. Advent calendars must be in store before.</t>
         </is>
@@ -2625,73 +2474,68 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Juleferie (skole)</t>
+          <t>Christmas school break (Juleferie)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Christmas school break</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
           <t>Season &amp; holidays</t>
         </is>
       </c>
+      <c r="C31" s="2" t="n">
+        <v>46375</v>
+      </c>
       <c r="D31" s="2" t="n">
-        <v>46375</v>
-      </c>
-      <c r="E31" s="2" t="n">
         <v>46390</v>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Yes — range</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Yes — range</t>
+          <t>All of Norway</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
           <t>Travel, Kids &amp; family, Food &amp; drink, Retail</t>
         </is>
       </c>
+      <c r="H31" s="2" t="n">
+        <v>46262</v>
+      </c>
       <c r="I31" s="2" t="n">
-        <v>46262</v>
+        <v>46304</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>46304</v>
+        <v>46332</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>46332</v>
-      </c>
-      <c r="L31" s="2" t="n">
         <v>46367</v>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>observed</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>observed</t>
+          <t>19 Dec → 3 Jan (+1 y)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>19 Dec → 3 Jan (+1 y)</t>
+          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
-        <is>
-          <t>https://lovdata.no/dokument/NL/lov/2023-06-09-30</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
         <is>
           <t>Set locally; typically from the weekend before Christmas to the first working days of January (Oslo: 21 Dec 2026 – 1 Jan 2027; 20 Dec 2027 – 3 Jan 2028). Shown as ~19 Dec – ~3 Jan.</t>
         </is>
@@ -2700,284 +2544,264 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Julaften</t>
+          <t>Christmas Eve (Julaften)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Christmas Eve</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
           <t>Cultural moment</t>
         </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>46380</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>46380</v>
       </c>
-      <c r="E32" s="2" t="n">
-        <v>46380</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
           <t>Retail, Food &amp; drink, Kids &amp; family, Alcohol-free</t>
         </is>
       </c>
+      <c r="H32" s="2" t="n">
+        <v>46268</v>
+      </c>
       <c r="I32" s="2" t="n">
-        <v>46268</v>
+        <v>46310</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>46310</v>
+        <v>46338</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>46338</v>
-      </c>
-      <c r="L32" s="2" t="n">
         <v>46373</v>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>24 Dec</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>24 Dec</t>
+          <t>https://snl.no/julaften</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>https://snl.no/julaften</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>The main Norwegian Christmas celebration (ribbe/pinnekjøtt, presents in the evening). Not a helligdag under helligdagsfredloven § 2, but shops close early.</t>
+          <t>The main Norwegian Christmas celebration (pork rib or cured lamb rib — ribbe or pinnekjøtt — and presents in the evening). Not a public holiday under helligdagsfredloven § 2, but shops close early.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1. juledag</t>
+          <t>Christmas Day (1. juledag)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Christmas Day</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>46381</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>46381</v>
       </c>
-      <c r="E33" s="2" t="n">
-        <v>46381</v>
-      </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
           <t>Food &amp; drink, Kids &amp; family</t>
         </is>
       </c>
+      <c r="H33" s="2" t="n">
+        <v>46269</v>
+      </c>
       <c r="I33" s="2" t="n">
-        <v>46269</v>
+        <v>46311</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>46311</v>
+        <v>46339</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>46339</v>
-      </c>
-      <c r="L33" s="2" t="n">
         <v>46374</v>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>25 Dec</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>25 Dec</t>
+          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>Helligdag under helligdagsfredloven § 2.</t>
+          <t>Public holiday (helligdag) under the Public Holidays Act (helligdagsfredloven) § 2.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2. juledag</t>
+          <t>Boxing Day (2. juledag)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Boxing Day</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
           <t>Public holiday</t>
         </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>46382</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>46382</v>
       </c>
-      <c r="E34" s="2" t="n">
-        <v>46382</v>
-      </c>
-      <c r="F34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
           <t>Food &amp; drink</t>
         </is>
       </c>
+      <c r="H34" s="2" t="n">
+        <v>46269</v>
+      </c>
       <c r="I34" s="2" t="n">
-        <v>46269</v>
+        <v>46311</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>46311</v>
+        <v>46339</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>46339</v>
-      </c>
-      <c r="L34" s="2" t="n">
         <v>46374</v>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>official</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>26 Dec</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>26 Dec</t>
+          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>https://lovdata.no/dokument/NL/lov/1995-02-24-12</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>Helligdag under helligdagsfredloven § 2.</t>
+          <t>Public holiday (helligdag) under the Public Holidays Act (helligdagsfredloven) § 2.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Nyttårsaften</t>
+          <t>New Year's Eve (Nyttårsaften)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>New Year's Eve</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
           <t>Cultural moment</t>
         </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>46387</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>46387</v>
       </c>
-      <c r="E35" s="2" t="n">
-        <v>46387</v>
-      </c>
-      <c r="F35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>All of Norway</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Hele landet</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
           <t>Food &amp; drink, Fashion, Alcohol-free</t>
         </is>
       </c>
+      <c r="H35" s="2" t="n">
+        <v>46275</v>
+      </c>
       <c r="I35" s="2" t="n">
-        <v>46275</v>
+        <v>46317</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>46317</v>
+        <v>46345</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>46345</v>
-      </c>
-      <c r="L35" s="2" t="n">
         <v>46380</v>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>late start</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>late start</t>
+          <t>convention</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>convention</t>
+          <t>31 Dec</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>31 Dec</t>
+          <t>https://snl.no/nytt%C3%A5rsaften</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>https://snl.no/nytt%C3%A5rsaften</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>Party food, fireworks, party wear. Not a helligdag.</t>
+          <t>Party food, fireworks, party wear. Not a public holiday.</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2819,7 @@
   <dimension ref="A1:G137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -3044,7 +2868,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nyttårsdag</t>
+          <t>New Year's Day (Nyttårsdag)</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -3071,7 +2895,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Nyttårsdag</t>
+          <t>New Year's Day (Nyttårsdag)</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -3098,7 +2922,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nyttårsdag</t>
+          <t>New Year's Day (Nyttårsdag)</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -3125,7 +2949,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Nyttårsdag</t>
+          <t>New Year's Day (Nyttårsdag)</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -3154,7 +2978,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tørrlagt januar (Dry January)</t>
+          <t>Dry January (Tørrlagt januar)</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -3181,7 +3005,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tørrlagt januar (Dry January)</t>
+          <t>Dry January (Tørrlagt januar)</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -3208,7 +3032,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tørrlagt januar (Dry January)</t>
+          <t>Dry January (Tørrlagt januar)</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -3235,7 +3059,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tørrlagt januar (Dry January)</t>
+          <t>Dry January (Tørrlagt januar)</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -3264,7 +3088,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Morsdag</t>
+          <t>Mother's Day, Norway (Morsdag)</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -3293,7 +3117,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Morsdag</t>
+          <t>Mother's Day, Norway (Morsdag)</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
@@ -3322,7 +3146,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Morsdag</t>
+          <t>Mother's Day, Norway (Morsdag)</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -3351,7 +3175,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Morsdag</t>
+          <t>Mother's Day, Norway (Morsdag)</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
@@ -3380,7 +3204,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Valentinsdagen</t>
+          <t>Valentine's Day (Valentinsdagen)</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -3409,7 +3233,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Valentinsdagen</t>
+          <t>Valentine's Day (Valentinsdagen)</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
@@ -3438,7 +3262,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Valentinsdagen</t>
+          <t>Valentine's Day (Valentinsdagen)</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -3467,7 +3291,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Valentinsdagen</t>
+          <t>Valentine's Day (Valentinsdagen)</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
@@ -3496,7 +3320,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Fastelavnssøndag</t>
+          <t>Shrovetide Sunday (Fastelavnssøndag)</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -3525,7 +3349,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Fastelavnssøndag</t>
+          <t>Shrovetide Sunday (Fastelavnssøndag)</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
@@ -3554,7 +3378,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Fastelavnssøndag</t>
+          <t>Shrovetide Sunday (Fastelavnssøndag)</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -3583,7 +3407,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Fastelavnssøndag</t>
+          <t>Shrovetide Sunday (Fastelavnssøndag)</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -3612,7 +3436,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Vinterferie</t>
+          <t>Winter school break (Vinterferie)</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -3639,7 +3463,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Vinterferie</t>
+          <t>Winter school break (Vinterferie)</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
@@ -3666,7 +3490,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Vinterferie</t>
+          <t>Winter school break (Vinterferie)</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -3693,7 +3517,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Vinterferie</t>
+          <t>Winter school break (Vinterferie)</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
@@ -3720,7 +3544,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Påskeferie</t>
+          <t>Easter school break (Påskeferie)</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -3749,7 +3573,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Påskeferie</t>
+          <t>Easter school break (Påskeferie)</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
@@ -3778,7 +3602,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Påskeferie</t>
+          <t>Easter school break (Påskeferie)</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -3807,7 +3631,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Påskeferie</t>
+          <t>Easter school break (Påskeferie)</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
@@ -3836,7 +3660,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Skjærtorsdag</t>
+          <t>Maundy Thursday (Skjærtorsdag)</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -3863,7 +3687,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Skjærtorsdag</t>
+          <t>Maundy Thursday (Skjærtorsdag)</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
@@ -3890,7 +3714,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Skjærtorsdag</t>
+          <t>Maundy Thursday (Skjærtorsdag)</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -3917,7 +3741,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Skjærtorsdag</t>
+          <t>Maundy Thursday (Skjærtorsdag)</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
@@ -3944,7 +3768,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Langfredag</t>
+          <t>Good Friday (Langfredag)</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -3971,7 +3795,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Langfredag</t>
+          <t>Good Friday (Langfredag)</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
@@ -3998,7 +3822,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Langfredag</t>
+          <t>Good Friday (Langfredag)</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -4025,7 +3849,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Langfredag</t>
+          <t>Good Friday (Langfredag)</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
@@ -4052,7 +3876,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Påskedag</t>
+          <t>Easter Sunday (Påskedag)</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -4081,7 +3905,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Påskedag</t>
+          <t>Easter Sunday (Påskedag)</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
@@ -4110,7 +3934,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Påskedag</t>
+          <t>Easter Sunday (Påskedag)</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -4139,7 +3963,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Påskedag</t>
+          <t>Easter Sunday (Påskedag)</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
@@ -4168,7 +3992,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2. påskedag</t>
+          <t>Easter Monday (2. påskedag)</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -4195,7 +4019,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2. påskedag</t>
+          <t>Easter Monday (2. påskedag)</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
@@ -4222,7 +4046,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2. påskedag</t>
+          <t>Easter Monday (2. påskedag)</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -4249,7 +4073,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2. påskedag</t>
+          <t>Easter Monday (2. påskedag)</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
@@ -4276,7 +4100,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Russetiden</t>
+          <t>Russ celebration season (Russetiden)</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -4303,7 +4127,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Russetiden</t>
+          <t>Russ celebration season (Russetiden)</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
@@ -4330,7 +4154,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Russetiden</t>
+          <t>Russ celebration season (Russetiden)</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -4357,7 +4181,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Russetiden</t>
+          <t>Russ celebration season (Russetiden)</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
@@ -4384,7 +4208,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1. mai — Arbeidernes dag</t>
+          <t>May Day (1. mai — Arbeidernes dag)</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -4411,7 +4235,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1. mai — Arbeidernes dag</t>
+          <t>May Day (1. mai — Arbeidernes dag)</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
@@ -4438,7 +4262,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1. mai — Arbeidernes dag</t>
+          <t>May Day (1. mai — Arbeidernes dag)</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -4465,7 +4289,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1. mai — Arbeidernes dag</t>
+          <t>May Day (1. mai — Arbeidernes dag)</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
@@ -4492,7 +4316,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Kristi himmelfartsdag</t>
+          <t>Ascension Day (Kristi himmelfartsdag)</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -4519,7 +4343,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Kristi himmelfartsdag</t>
+          <t>Ascension Day (Kristi himmelfartsdag)</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
@@ -4546,7 +4370,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Kristi himmelfartsdag</t>
+          <t>Ascension Day (Kristi himmelfartsdag)</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -4575,7 +4399,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Kristi himmelfartsdag</t>
+          <t>Ascension Day (Kristi himmelfartsdag)</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
@@ -4602,7 +4426,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>17. mai — Grunnlovsdagen</t>
+          <t>Constitution Day (17. mai — Grunnlovsdagen)</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -4631,7 +4455,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>17. mai — Grunnlovsdagen</t>
+          <t>Constitution Day (17. mai — Grunnlovsdagen)</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
@@ -4660,7 +4484,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>17. mai — Grunnlovsdagen</t>
+          <t>Constitution Day (17. mai — Grunnlovsdagen)</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -4689,7 +4513,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>17. mai — Grunnlovsdagen</t>
+          <t>Constitution Day (17. mai — Grunnlovsdagen)</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
@@ -4718,7 +4542,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Pinsedag</t>
+          <t>Whit Sunday (Pinsedag)</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -4747,7 +4571,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Pinsedag</t>
+          <t>Whit Sunday (Pinsedag)</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
@@ -4776,7 +4600,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Pinsedag</t>
+          <t>Whit Sunday (Pinsedag)</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -4805,7 +4629,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Pinsedag</t>
+          <t>Whit Sunday (Pinsedag)</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
@@ -4834,7 +4658,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2. pinsedag</t>
+          <t>Whit Monday (2. pinsedag)</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -4861,7 +4685,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2. pinsedag</t>
+          <t>Whit Monday (2. pinsedag)</t>
         </is>
       </c>
       <c r="B67" s="2" t="n">
@@ -4888,7 +4712,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2. pinsedag</t>
+          <t>Whit Monday (2. pinsedag)</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -4915,7 +4739,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2. pinsedag</t>
+          <t>Whit Monday (2. pinsedag)</t>
         </is>
       </c>
       <c r="B69" s="2" t="n">
@@ -4942,7 +4766,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Skoleslutt</t>
+          <t>Last day of school (Skoleslutt)</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -4969,7 +4793,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Skoleslutt</t>
+          <t>Last day of school (Skoleslutt)</t>
         </is>
       </c>
       <c r="B71" s="2" t="n">
@@ -4996,7 +4820,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Skoleslutt</t>
+          <t>Last day of school (Skoleslutt)</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -5023,7 +4847,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Skoleslutt</t>
+          <t>Last day of school (Skoleslutt)</t>
         </is>
       </c>
       <c r="B73" s="2" t="n">
@@ -5050,7 +4874,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Sankthansaften</t>
+          <t>Midsummer Eve (Sankthansaften)</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
@@ -5077,7 +4901,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Sankthansaften</t>
+          <t>Midsummer Eve (Sankthansaften)</t>
         </is>
       </c>
       <c r="B75" s="2" t="n">
@@ -5104,7 +4928,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Sankthansaften</t>
+          <t>Midsummer Eve (Sankthansaften)</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -5131,7 +4955,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Sankthansaften</t>
+          <t>Midsummer Eve (Sankthansaften)</t>
         </is>
       </c>
       <c r="B77" s="2" t="n">
@@ -5158,7 +4982,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Fellesferie</t>
+          <t>Collective summer holiday (Fellesferie)</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -5185,7 +5009,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Fellesferie</t>
+          <t>Collective summer holiday (Fellesferie)</t>
         </is>
       </c>
       <c r="B79" s="2" t="n">
@@ -5212,7 +5036,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Fellesferie</t>
+          <t>Collective summer holiday (Fellesferie)</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -5241,7 +5065,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Fellesferie</t>
+          <t>Collective summer holiday (Fellesferie)</t>
         </is>
       </c>
       <c r="B81" s="2" t="n">
@@ -5268,7 +5092,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Skolestart</t>
+          <t>Back to school (Skolestart)</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -5295,7 +5119,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Skolestart</t>
+          <t>Back to school (Skolestart)</t>
         </is>
       </c>
       <c r="B83" s="2" t="n">
@@ -5322,7 +5146,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Skolestart</t>
+          <t>Back to school (Skolestart)</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -5349,7 +5173,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Skolestart</t>
+          <t>Back to school (Skolestart)</t>
         </is>
       </c>
       <c r="B85" s="2" t="n">
@@ -5376,7 +5200,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Høstferie</t>
+          <t>Autumn school break (Høstferie)</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -5403,7 +5227,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Høstferie</t>
+          <t>Autumn school break (Høstferie)</t>
         </is>
       </c>
       <c r="B87" s="2" t="n">
@@ -5430,7 +5254,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Høstferie</t>
+          <t>Autumn school break (Høstferie)</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -5457,7 +5281,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Høstferie</t>
+          <t>Autumn school break (Høstferie)</t>
         </is>
       </c>
       <c r="B89" s="2" t="n">
@@ -5600,7 +5424,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Farsdag</t>
+          <t>Father's Day, Norway (Farsdag)</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -5629,7 +5453,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Farsdag</t>
+          <t>Father's Day, Norway (Farsdag)</t>
         </is>
       </c>
       <c r="B95" s="2" t="n">
@@ -5658,7 +5482,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Farsdag</t>
+          <t>Father's Day, Norway (Farsdag)</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
@@ -5687,7 +5511,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Farsdag</t>
+          <t>Father's Day, Norway (Farsdag)</t>
         </is>
       </c>
       <c r="B97" s="2" t="n">
@@ -5716,7 +5540,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Julebordsesongen</t>
+          <t>Christmas-party season (Julebordsesongen)</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -5743,7 +5567,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Julebordsesongen</t>
+          <t>Christmas-party season (Julebordsesongen)</t>
         </is>
       </c>
       <c r="B99" s="2" t="n">
@@ -5770,7 +5594,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Julebordsesongen</t>
+          <t>Christmas-party season (Julebordsesongen)</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
@@ -5797,7 +5621,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Julebordsesongen</t>
+          <t>Christmas-party season (Julebordsesongen)</t>
         </is>
       </c>
       <c r="B101" s="2" t="n">
@@ -5932,7 +5756,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Julehandelen</t>
+          <t>Christmas shopping season (Julehandelen)</t>
         </is>
       </c>
       <c r="B106" s="2" t="n">
@@ -5959,7 +5783,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Julehandelen</t>
+          <t>Christmas shopping season (Julehandelen)</t>
         </is>
       </c>
       <c r="B107" s="2" t="n">
@@ -5986,7 +5810,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Julehandelen</t>
+          <t>Christmas shopping season (Julehandelen)</t>
         </is>
       </c>
       <c r="B108" s="2" t="n">
@@ -6013,7 +5837,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Julehandelen</t>
+          <t>Christmas shopping season (Julehandelen)</t>
         </is>
       </c>
       <c r="B109" s="2" t="n">
@@ -6148,7 +5972,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>1. søndag i advent</t>
+          <t>First Sunday of Advent (1. søndag i advent)</t>
         </is>
       </c>
       <c r="B114" s="2" t="n">
@@ -6177,7 +6001,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>1. søndag i advent</t>
+          <t>First Sunday of Advent (1. søndag i advent)</t>
         </is>
       </c>
       <c r="B115" s="2" t="n">
@@ -6206,7 +6030,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>1. søndag i advent</t>
+          <t>First Sunday of Advent (1. søndag i advent)</t>
         </is>
       </c>
       <c r="B116" s="2" t="n">
@@ -6235,7 +6059,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>1. søndag i advent</t>
+          <t>First Sunday of Advent (1. søndag i advent)</t>
         </is>
       </c>
       <c r="B117" s="2" t="n">
@@ -6264,7 +6088,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Juleferie (skole)</t>
+          <t>Christmas school break (Juleferie)</t>
         </is>
       </c>
       <c r="B118" s="2" t="n">
@@ -6293,7 +6117,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Juleferie (skole)</t>
+          <t>Christmas school break (Juleferie)</t>
         </is>
       </c>
       <c r="B119" s="2" t="n">
@@ -6322,7 +6146,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Juleferie (skole)</t>
+          <t>Christmas school break (Juleferie)</t>
         </is>
       </c>
       <c r="B120" s="2" t="n">
@@ -6351,7 +6175,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Juleferie (skole)</t>
+          <t>Christmas school break (Juleferie)</t>
         </is>
       </c>
       <c r="B121" s="2" t="n">
@@ -6380,7 +6204,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Julaften</t>
+          <t>Christmas Eve (Julaften)</t>
         </is>
       </c>
       <c r="B122" s="2" t="n">
@@ -6407,7 +6231,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Julaften</t>
+          <t>Christmas Eve (Julaften)</t>
         </is>
       </c>
       <c r="B123" s="2" t="n">
@@ -6434,7 +6258,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Julaften</t>
+          <t>Christmas Eve (Julaften)</t>
         </is>
       </c>
       <c r="B124" s="2" t="n">
@@ -6461,7 +6285,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Julaften</t>
+          <t>Christmas Eve (Julaften)</t>
         </is>
       </c>
       <c r="B125" s="2" t="n">
@@ -6488,7 +6312,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>1. juledag</t>
+          <t>Christmas Day (1. juledag)</t>
         </is>
       </c>
       <c r="B126" s="2" t="n">
@@ -6515,7 +6339,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>1. juledag</t>
+          <t>Christmas Day (1. juledag)</t>
         </is>
       </c>
       <c r="B127" s="2" t="n">
@@ -6542,7 +6366,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>1. juledag</t>
+          <t>Christmas Day (1. juledag)</t>
         </is>
       </c>
       <c r="B128" s="2" t="n">
@@ -6569,7 +6393,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>1. juledag</t>
+          <t>Christmas Day (1. juledag)</t>
         </is>
       </c>
       <c r="B129" s="2" t="n">
@@ -6596,7 +6420,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2. juledag</t>
+          <t>Boxing Day (2. juledag)</t>
         </is>
       </c>
       <c r="B130" s="2" t="n">
@@ -6625,7 +6449,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2. juledag</t>
+          <t>Boxing Day (2. juledag)</t>
         </is>
       </c>
       <c r="B131" s="2" t="n">
@@ -6654,7 +6478,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2. juledag</t>
+          <t>Boxing Day (2. juledag)</t>
         </is>
       </c>
       <c r="B132" s="2" t="n">
@@ -6683,7 +6507,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2. juledag</t>
+          <t>Boxing Day (2. juledag)</t>
         </is>
       </c>
       <c r="B133" s="2" t="n">
@@ -6712,7 +6536,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Nyttårsaften</t>
+          <t>New Year's Eve (Nyttårsaften)</t>
         </is>
       </c>
       <c r="B134" s="2" t="n">
@@ -6739,7 +6563,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Nyttårsaften</t>
+          <t>New Year's Eve (Nyttårsaften)</t>
         </is>
       </c>
       <c r="B135" s="2" t="n">
@@ -6766,7 +6590,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Nyttårsaften</t>
+          <t>New Year's Eve (Nyttårsaften)</t>
         </is>
       </c>
       <c r="B136" s="2" t="n">
@@ -6793,7 +6617,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Nyttårsaften</t>
+          <t>New Year's Eve (Nyttårsaften)</t>
         </is>
       </c>
       <c r="B137" s="2" t="n">
@@ -6833,9 +6657,9 @@
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
@@ -6932,7 +6756,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Påskeferie</t>
+          <t>Easter school break (Påskeferie)</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -6940,7 +6764,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Hele landet</t>
+          <t>All of Norway</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -6992,7 +6816,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>17. mai — Grunnlovsdagen</t>
+          <t>Constitution Day (17. mai — Grunnlovsdagen)</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -7000,7 +6824,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Hele landet</t>
+          <t>All of Norway</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -7060,7 +6884,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Hele landet</t>
+          <t>All of Norway</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -7376,7 +7200,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dates are computed from rules in the moments library. Moments marked 'varies locally' show a national range — check the kommune's skolerute. Lead times are editable planning conventions, not research.</t>
+          <t>Dates are computed from rules in the moments library. Moments marked 'varies locally' show a national range — check the municipality's school calendar (skolerute). Lead times are editable planning conventions, not research.</t>
         </is>
       </c>
     </row>

</xml_diff>